<commit_message>
batch 3: rest/b2b effect shipped into sims (+alignment bugfix); tank/familiarity/team-HFA/heavy-hockey nulls; relative-age + SO documented
</commit_message>
<xml_diff>
--- a/output/nhl_2026_27_projections_v3.xlsx
+++ b/output/nhl_2026_27_projections_v3.xlsx
@@ -678,24 +678,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Carolina Hurricanes</t>
+          <t>Colorado Avalanche</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>107.6031</v>
+        <v>107.5517</v>
       </c>
       <c r="F2" t="n">
-        <v>12.63599371730306</v>
+        <v>12.69404746304737</v>
       </c>
       <c r="G2" t="n">
         <v>86</v>
@@ -707,42 +707,42 @@
         <v>128</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8436</v>
+        <v>0.8724</v>
       </c>
       <c r="K2" t="n">
-        <v>0.4137</v>
+        <v>0.3469</v>
       </c>
       <c r="L2" t="n">
-        <v>0.192</v>
+        <v>0.1866</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1132</v>
+        <v>0.1023</v>
       </c>
       <c r="N2" t="n">
-        <v>8.287039933520225</v>
+        <v>10.43058285193634</v>
       </c>
       <c r="O2" t="n">
-        <v>-1.8</v>
+        <v>-6.5</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>+783</t>
+          <t>+878</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>14.86116182018452</v>
+        <v>14.53741765167042</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.1669627848400201</v>
+        <v>-1.301203426971305</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.2526154518856217</v>
+        <v>-1.546832861222726</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2384111455252166</v>
+        <v>0.9853425117174447</v>
       </c>
       <c r="U2" t="n">
-        <v>-1.298489907419239</v>
+        <v>1.035664354688619</v>
       </c>
     </row>
     <row r="3">
@@ -751,24 +751,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Colorado Avalanche</t>
+          <t>Carolina Hurricanes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>107.416</v>
+        <v>107.5266</v>
       </c>
       <c r="F3" t="n">
-        <v>12.75622264314998</v>
+        <v>12.5644211529179</v>
       </c>
       <c r="G3" t="n">
         <v>86</v>
@@ -780,42 +780,42 @@
         <v>128</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8702</v>
+        <v>0.8454</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3424</v>
+        <v>0.4146</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1886</v>
+        <v>0.1933</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1036</v>
+        <v>0.1129</v>
       </c>
       <c r="N3" t="n">
-        <v>10.43058285193634</v>
+        <v>8.287039933520225</v>
       </c>
       <c r="O3" t="n">
-        <v>-6.5</v>
+        <v>-1.8</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>+865</t>
+          <t>+786</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>14.53741765167042</v>
+        <v>14.86116182018452</v>
       </c>
       <c r="R3" t="n">
-        <v>-1.301203426971305</v>
+        <v>-0.1669627848400201</v>
       </c>
       <c r="S3" t="n">
-        <v>-1.546832861222726</v>
+        <v>-0.2526154518856217</v>
       </c>
       <c r="T3" t="n">
-        <v>0.9853425117174447</v>
+        <v>0.2384111455252166</v>
       </c>
       <c r="U3" t="n">
-        <v>1.035664354688619</v>
+        <v>-1.298489907419239</v>
       </c>
     </row>
     <row r="4">
@@ -838,31 +838,31 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>105.0989</v>
+        <v>105.2254</v>
       </c>
       <c r="F4" t="n">
-        <v>12.80805697295036</v>
+        <v>12.73178717543095</v>
       </c>
       <c r="G4" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H4" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I4" t="n">
         <v>125</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8547</v>
+        <v>0.8583</v>
       </c>
       <c r="K4" t="n">
-        <v>0.4173</v>
+        <v>0.4208</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1711</v>
+        <v>0.1691</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0896</v>
+        <v>0.0895</v>
       </c>
       <c r="N4" t="n">
         <v>9.436252802325914</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>+1016</t>
+          <t>+1017</t>
         </is>
       </c>
       <c r="Q4" t="n">
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>104.481</v>
+        <v>104.6473</v>
       </c>
       <c r="F5" t="n">
-        <v>12.80072751301606</v>
+        <v>12.77810747775551</v>
       </c>
       <c r="G5" t="n">
         <v>83</v>
@@ -926,16 +926,16 @@
         <v>125</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8128</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2499</v>
+        <v>0.2534</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1513</v>
+        <v>0.1509</v>
       </c>
       <c r="M5" t="n">
-        <v>0.079</v>
+        <v>0.0781</v>
       </c>
       <c r="N5" t="n">
         <v>9.85275482151591</v>
@@ -945,7 +945,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>+1166</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="Q5" t="n">
@@ -970,12 +970,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tampa Bay Lightning</t>
+          <t>Montreal Canadiens</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBL</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -984,57 +984,57 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>102.882</v>
+        <v>103.2097</v>
       </c>
       <c r="F6" t="n">
-        <v>13.08393652306117</v>
+        <v>12.67461993548725</v>
       </c>
       <c r="G6" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H6" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I6" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J6" t="n">
-        <v>0.7282999999999999</v>
+        <v>0.7475000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2399</v>
+        <v>0.2383</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1235</v>
+        <v>0.1173</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0677</v>
+        <v>0.0592</v>
       </c>
       <c r="N6" t="n">
-        <v>11.95676267158673</v>
+        <v>8.510549067215697</v>
       </c>
       <c r="O6" t="n">
-        <v>-6.7</v>
+        <v>-2.5</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>+1377</t>
+          <t>+1589</t>
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>9.436735107173774</v>
+        <v>1.740788541281878</v>
       </c>
       <c r="R6" t="n">
-        <v>-0.8022613128825858</v>
+        <v>2.510899193633914</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.8994067827698127</v>
+        <v>2.196737059056645</v>
       </c>
       <c r="T6" t="n">
-        <v>2.111485424037829</v>
+        <v>0.6120765889048018</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5100934026557666</v>
+        <v>1.804633765882705</v>
       </c>
     </row>
     <row r="7">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Montreal Canadiens</t>
+          <t>Tampa Bay Lightning</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>TBL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>102.2868</v>
+        <v>102.8115</v>
       </c>
       <c r="F7" t="n">
-        <v>12.77859440656525</v>
+        <v>13.02534965839199</v>
       </c>
       <c r="G7" t="n">
         <v>81</v>
@@ -1069,45 +1069,45 @@
         <v>103</v>
       </c>
       <c r="I7" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7165</v>
+        <v>0.7295</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2122</v>
+        <v>0.2388</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1138</v>
+        <v>0.1247</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0613</v>
+        <v>0.0692</v>
       </c>
       <c r="N7" t="n">
-        <v>8.510549067215697</v>
+        <v>11.95676267158673</v>
       </c>
       <c r="O7" t="n">
-        <v>-2.5</v>
+        <v>-6.7</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>+1531</t>
+          <t>+1345</t>
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>1.740788541281878</v>
+        <v>9.436735107173774</v>
       </c>
       <c r="R7" t="n">
-        <v>2.510899193633914</v>
+        <v>-0.8022613128825858</v>
       </c>
       <c r="S7" t="n">
-        <v>2.196737059056645</v>
+        <v>-0.8994067827698127</v>
       </c>
       <c r="T7" t="n">
-        <v>0.6120765889048018</v>
+        <v>2.111485424037829</v>
       </c>
       <c r="U7" t="n">
-        <v>1.804633765882705</v>
+        <v>0.5100934026557666</v>
       </c>
     </row>
     <row r="8">
@@ -1116,24 +1116,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ottawa Senators</t>
+          <t>Edmonton Oilers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>EDM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>101.9931</v>
+        <v>101.6318</v>
       </c>
       <c r="F8" t="n">
-        <v>12.77485702805353</v>
+        <v>12.96984388668748</v>
       </c>
       <c r="G8" t="n">
         <v>80</v>
@@ -1145,42 +1145,42 @@
         <v>123</v>
       </c>
       <c r="J8" t="n">
-        <v>0.7091</v>
+        <v>0.783</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2076</v>
+        <v>0.2956</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1091</v>
+        <v>0.1245</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0544</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>7.085134171727478</v>
+        <v>11.11131222666323</v>
       </c>
       <c r="O8" t="n">
-        <v>-4.1</v>
+        <v>2.7</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>+1738</t>
+          <t>+1470</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>8.451268172646309</v>
+        <v>3.210989299173198</v>
       </c>
       <c r="R8" t="n">
-        <v>1.77019449892022</v>
+        <v>-1.056838272229703</v>
       </c>
       <c r="S8" t="n">
-        <v>1.156408289279054</v>
+        <v>-0.8014174971800627</v>
       </c>
       <c r="T8" t="n">
-        <v>0.3775057526043846</v>
+        <v>1.235756684107004</v>
       </c>
       <c r="U8" t="n">
-        <v>-2.897413578334854</v>
+        <v>3.501549285384193</v>
       </c>
     </row>
     <row r="9">
@@ -1189,24 +1189,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Edmonton Oilers</t>
+          <t>Ottawa Senators</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>101.821</v>
+        <v>101.283</v>
       </c>
       <c r="F9" t="n">
-        <v>13.03574133124793</v>
+        <v>12.75202620830281</v>
       </c>
       <c r="G9" t="n">
         <v>80</v>
@@ -1215,45 +1215,45 @@
         <v>102</v>
       </c>
       <c r="I9" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7891</v>
+        <v>0.6962</v>
       </c>
       <c r="K9" t="n">
-        <v>0.3019</v>
+        <v>0.1967</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1269</v>
+        <v>0.107</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0644</v>
+        <v>0.0549</v>
       </c>
       <c r="N9" t="n">
-        <v>11.11131222666323</v>
+        <v>7.085134171727478</v>
       </c>
       <c r="O9" t="n">
-        <v>2.7</v>
+        <v>-4.1</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>+1453</t>
+          <t>+1721</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>3.210989299173198</v>
+        <v>8.451268172646309</v>
       </c>
       <c r="R9" t="n">
-        <v>-1.056838272229703</v>
+        <v>1.77019449892022</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.8014174971800627</v>
+        <v>1.156408289279054</v>
       </c>
       <c r="T9" t="n">
-        <v>1.235756684107004</v>
+        <v>0.3775057526043846</v>
       </c>
       <c r="U9" t="n">
-        <v>3.501549285384193</v>
+        <v>-2.897413578334854</v>
       </c>
     </row>
     <row r="10">
@@ -1276,13 +1276,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>100.1821</v>
+        <v>100.2607</v>
       </c>
       <c r="F10" t="n">
-        <v>13.00620835353538</v>
+        <v>12.96781986091704</v>
       </c>
       <c r="G10" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H10" t="n">
         <v>101</v>
@@ -1291,16 +1291,16 @@
         <v>121</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6656</v>
+        <v>0.6708</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1955</v>
+        <v>0.1928</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0917</v>
+        <v>0.0911</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0486</v>
+        <v>0.0472</v>
       </c>
       <c r="N10" t="n">
         <v>8.112523146305424</v>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>+1958</t>
+          <t>+2019</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -1349,10 +1349,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>99.093</v>
+        <v>98.7401</v>
       </c>
       <c r="F11" t="n">
-        <v>13.06614034067981</v>
+        <v>13.04902983780675</v>
       </c>
       <c r="G11" t="n">
         <v>77</v>
@@ -1364,16 +1364,16 @@
         <v>120</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6806</v>
+        <v>0.6701</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1402</v>
+        <v>0.1357</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0851</v>
+        <v>0.0881</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0386</v>
+        <v>0.0402</v>
       </c>
       <c r="N11" t="n">
         <v>8.309178835527998</v>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>+2491</t>
+          <t>+2388</t>
         </is>
       </c>
       <c r="Q11" t="n">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>97.38849999999999</v>
+        <v>96.9571</v>
       </c>
       <c r="F12" t="n">
-        <v>13.09418624891796</v>
+        <v>13.10187106838368</v>
       </c>
       <c r="G12" t="n">
         <v>76</v>
@@ -1434,19 +1434,19 @@
         <v>97</v>
       </c>
       <c r="I12" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5673</v>
+        <v>0.5589</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1276</v>
+        <v>0.1232</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0649</v>
+        <v>0.0646</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0329</v>
+        <v>0.0346</v>
       </c>
       <c r="N12" t="n">
         <v>7.27216984942758</v>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>+2940</t>
+          <t>+2790</t>
         </is>
       </c>
       <c r="Q12" t="n">
@@ -1495,10 +1495,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>97.0558</v>
+        <v>96.8592</v>
       </c>
       <c r="F13" t="n">
-        <v>13.07049234485885</v>
+        <v>13.04591870891031</v>
       </c>
       <c r="G13" t="n">
         <v>75</v>
@@ -1510,16 +1510,16 @@
         <v>118</v>
       </c>
       <c r="J13" t="n">
-        <v>0.6249</v>
+        <v>0.6221</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1123</v>
+        <v>0.1066</v>
       </c>
       <c r="L13" t="n">
-        <v>0.0665</v>
+        <v>0.0687</v>
       </c>
       <c r="M13" t="n">
-        <v>0.03</v>
+        <v>0.0321</v>
       </c>
       <c r="N13" t="n">
         <v>8.023130703542428</v>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>+3233</t>
+          <t>+3015</t>
         </is>
       </c>
       <c r="Q13" t="n">
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>95.0716</v>
+        <v>94.40779999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>13.21966525275657</v>
+        <v>13.11450716534247</v>
       </c>
       <c r="G14" t="n">
         <v>73</v>
@@ -1580,19 +1580,19 @@
         <v>95</v>
       </c>
       <c r="I14" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5041</v>
+        <v>0.488</v>
       </c>
       <c r="K14" t="n">
-        <v>0.0954</v>
+        <v>0.0867</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0496</v>
+        <v>0.0482</v>
       </c>
       <c r="M14" t="n">
-        <v>0.023</v>
+        <v>0.0229</v>
       </c>
       <c r="N14" t="n">
         <v>7.661371017102861</v>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>+4248</t>
+          <t>+4267</t>
         </is>
       </c>
       <c r="Q14" t="n">
@@ -1641,10 +1641,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>93.74379999999999</v>
+        <v>93.71129999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>13.23280288779466</v>
+        <v>13.21520398902897</v>
       </c>
       <c r="G15" t="n">
         <v>72</v>
@@ -1656,16 +1656,16 @@
         <v>115</v>
       </c>
       <c r="J15" t="n">
-        <v>0.4719</v>
+        <v>0.4801</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0927</v>
+        <v>0.0944</v>
       </c>
       <c r="L15" t="n">
-        <v>0.0443</v>
+        <v>0.0434</v>
       </c>
       <c r="M15" t="n">
-        <v>0.0202</v>
+        <v>0.0197</v>
       </c>
       <c r="N15" t="n">
         <v>6.130068512120818</v>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>+4850</t>
+          <t>+4976</t>
         </is>
       </c>
       <c r="Q15" t="n">
@@ -1714,10 +1714,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>93.7159</v>
+        <v>93.3905</v>
       </c>
       <c r="F16" t="n">
-        <v>13.07881847642492</v>
+        <v>13.01923806549295</v>
       </c>
       <c r="G16" t="n">
         <v>72</v>
@@ -1726,19 +1726,19 @@
         <v>94</v>
       </c>
       <c r="I16" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J16" t="n">
-        <v>0.4774</v>
+        <v>0.4709</v>
       </c>
       <c r="K16" t="n">
-        <v>0.08840000000000001</v>
+        <v>0.0857</v>
       </c>
       <c r="L16" t="n">
-        <v>0.044</v>
+        <v>0.0434</v>
       </c>
       <c r="M16" t="n">
-        <v>0.0193</v>
+        <v>0.0184</v>
       </c>
       <c r="N16" t="n">
         <v>7.139596880634292</v>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>+5081</t>
+          <t>+5335</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -1787,10 +1787,10 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>92.83580000000001</v>
+        <v>92.5158</v>
       </c>
       <c r="F17" t="n">
-        <v>13.22705310541185</v>
+        <v>13.19383030343378</v>
       </c>
       <c r="G17" t="n">
         <v>71</v>
@@ -1802,16 +1802,16 @@
         <v>114</v>
       </c>
       <c r="J17" t="n">
-        <v>0.4539</v>
+        <v>0.4445</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0813</v>
+        <v>0.0803</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0392</v>
+        <v>0.0388</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0199</v>
+        <v>0.0177</v>
       </c>
       <c r="N17" t="n">
         <v>9.661055316871911</v>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>+4925</t>
+          <t>+5550</t>
         </is>
       </c>
       <c r="Q17" t="n">
@@ -1860,31 +1860,31 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>91.96550000000001</v>
+        <v>92.41670000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>13.07311747021494</v>
+        <v>13.01610552393845</v>
       </c>
       <c r="G18" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H18" t="n">
         <v>92</v>
       </c>
       <c r="I18" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J18" t="n">
-        <v>0.4677</v>
+        <v>0.4747</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0559</v>
+        <v>0.0595</v>
       </c>
       <c r="L18" t="n">
-        <v>0.0366</v>
+        <v>0.0355</v>
       </c>
       <c r="M18" t="n">
-        <v>0.0133</v>
+        <v>0.014</v>
       </c>
       <c r="N18" t="n">
         <v>6.73886642624792</v>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>+7419</t>
+          <t>+7043</t>
         </is>
       </c>
       <c r="Q18" t="n">
@@ -1933,13 +1933,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>91.5638</v>
+        <v>91.6692</v>
       </c>
       <c r="F19" t="n">
-        <v>13.26660204547431</v>
+        <v>13.18906238125552</v>
       </c>
       <c r="G19" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H19" t="n">
         <v>92</v>
@@ -1948,16 +1948,16 @@
         <v>114</v>
       </c>
       <c r="J19" t="n">
-        <v>0.5052</v>
+        <v>0.5074</v>
       </c>
       <c r="K19" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.1009</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0387</v>
+        <v>0.0389</v>
       </c>
       <c r="M19" t="n">
-        <v>0.0163</v>
+        <v>0.0161</v>
       </c>
       <c r="N19" t="n">
         <v>8.389923070792923</v>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>+6035</t>
+          <t>+6111</t>
         </is>
       </c>
       <c r="Q19" t="n">
@@ -2006,10 +2006,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>91.4713</v>
+        <v>91.5787</v>
       </c>
       <c r="F20" t="n">
-        <v>13.24839342346197</v>
+        <v>13.17141430999316</v>
       </c>
       <c r="G20" t="n">
         <v>70</v>
@@ -2021,16 +2021,16 @@
         <v>113</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4593</v>
+        <v>0.4572</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0526</v>
+        <v>0.0527</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0365</v>
+        <v>0.037</v>
       </c>
       <c r="M20" t="n">
-        <v>0.0171</v>
+        <v>0.0164</v>
       </c>
       <c r="N20" t="n">
         <v>8.467264727101742</v>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>+5748</t>
+          <t>+5998</t>
         </is>
       </c>
       <c r="Q20" t="n">
@@ -2079,10 +2079,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>90.82340000000001</v>
+        <v>90.9911</v>
       </c>
       <c r="F21" t="n">
-        <v>13.13901350207011</v>
+        <v>13.10347247446603</v>
       </c>
       <c r="G21" t="n">
         <v>69</v>
@@ -2094,16 +2094,16 @@
         <v>112</v>
       </c>
       <c r="J21" t="n">
-        <v>0.3909</v>
+        <v>0.3969</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0577</v>
+        <v>0.0593</v>
       </c>
       <c r="L21" t="n">
-        <v>0.0301</v>
+        <v>0.0295</v>
       </c>
       <c r="M21" t="n">
-        <v>0.0128</v>
+        <v>0.0121</v>
       </c>
       <c r="N21" t="n">
         <v>8.08185262922734</v>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>+7712</t>
+          <t>+8164</t>
         </is>
       </c>
       <c r="Q21" t="n">
@@ -2138,71 +2138,71 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Toronto Maple Leafs</t>
+          <t>New York Rangers</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>89.83880000000001</v>
+        <v>89.48260000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>13.08096807321894</v>
+        <v>13.31862740013333</v>
       </c>
       <c r="G22" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H22" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I22" t="n">
         <v>111</v>
       </c>
       <c r="J22" t="n">
-        <v>0.3466</v>
+        <v>0.3515</v>
       </c>
       <c r="K22" t="n">
-        <v>0.044</v>
+        <v>0.0532</v>
       </c>
       <c r="L22" t="n">
-        <v>0.025</v>
+        <v>0.0234</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0103</v>
+        <v>0.0092</v>
       </c>
       <c r="N22" t="n">
-        <v>8.7101896414871</v>
+        <v>7.823147646950697</v>
       </c>
       <c r="O22" t="n">
-        <v>13.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>+9609</t>
+          <t>+10770</t>
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>-8.193380227493302</v>
+        <v>-4.799844584438726</v>
       </c>
       <c r="R22" t="n">
-        <v>2.580073488194848</v>
+        <v>-1.908540197038762</v>
       </c>
       <c r="S22" t="n">
-        <v>-0.7984428608114038</v>
+        <v>0.4458023315861614</v>
       </c>
       <c r="T22" t="n">
-        <v>0.09756098771463831</v>
+        <v>-0.1363557253125856</v>
       </c>
       <c r="U22" t="n">
-        <v>0.4100984906928617</v>
+        <v>0.8318037149568038</v>
       </c>
     </row>
     <row r="23">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Florida Panthers</t>
+          <t>Toronto Maple Leafs</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2225,57 +2225,57 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>89.3768</v>
+        <v>89.1717</v>
       </c>
       <c r="F23" t="n">
-        <v>13.16504286340761</v>
+        <v>13.08918453476681</v>
       </c>
       <c r="G23" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H23" t="n">
         <v>89</v>
       </c>
       <c r="I23" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J23" t="n">
-        <v>0.332</v>
+        <v>0.3325</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0463</v>
+        <v>0.0427</v>
       </c>
       <c r="L23" t="n">
-        <v>0.0249</v>
+        <v>0.0238</v>
       </c>
       <c r="M23" t="n">
-        <v>0.0102</v>
+        <v>0.01</v>
       </c>
       <c r="N23" t="n">
-        <v>9.184839315742089</v>
+        <v>8.7101896414871</v>
       </c>
       <c r="O23" t="n">
-        <v>-0.5</v>
+        <v>13.2</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>+9704</t>
+          <t>+9900</t>
         </is>
       </c>
       <c r="Q23" t="n">
-        <v>0.6979198033265082</v>
+        <v>-8.193380227493302</v>
       </c>
       <c r="R23" t="n">
-        <v>-2.218535999354475</v>
+        <v>2.580073488194848</v>
       </c>
       <c r="S23" t="n">
-        <v>0.3343300754021691</v>
+        <v>-0.7984428608114038</v>
       </c>
       <c r="T23" t="n">
-        <v>1.285179068259477</v>
+        <v>0.09756098771463831</v>
       </c>
       <c r="U23" t="n">
-        <v>-3.142967471019861</v>
+        <v>0.4100984906928617</v>
       </c>
     </row>
     <row r="24">
@@ -2284,71 +2284,71 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Winnipeg Jets</t>
+          <t>Florida Panthers</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>89.19759999999999</v>
+        <v>88.7985</v>
       </c>
       <c r="F24" t="n">
-        <v>13.03733682372077</v>
+        <v>13.10401729535366</v>
       </c>
       <c r="G24" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H24" t="n">
         <v>89</v>
       </c>
       <c r="I24" t="n">
-        <v>111</v>
+        <v>110.0499999999993</v>
       </c>
       <c r="J24" t="n">
-        <v>0.3867</v>
+        <v>0.3237</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0372</v>
+        <v>0.0444</v>
       </c>
       <c r="L24" t="n">
-        <v>0.0237</v>
+        <v>0.0255</v>
       </c>
       <c r="M24" t="n">
-        <v>0.0095</v>
+        <v>0.0113</v>
       </c>
       <c r="N24" t="n">
-        <v>8.140000216729245</v>
+        <v>9.184839315742089</v>
       </c>
       <c r="O24" t="n">
-        <v>-0.8</v>
+        <v>-0.5</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>+10426</t>
+          <t>+8750</t>
         </is>
       </c>
       <c r="Q24" t="n">
-        <v>-2.74817447802685</v>
+        <v>0.6979198033265082</v>
       </c>
       <c r="R24" t="n">
-        <v>-0.03608817469521482</v>
+        <v>-2.218535999354475</v>
       </c>
       <c r="S24" t="n">
-        <v>-2.183910751078082</v>
+        <v>0.3343300754021691</v>
       </c>
       <c r="T24" t="n">
-        <v>1.080791714011119</v>
+        <v>1.285179068259477</v>
       </c>
       <c r="U24" t="n">
-        <v>0.09443943429775073</v>
+        <v>-3.142967471019861</v>
       </c>
     </row>
     <row r="25">
@@ -2357,24 +2357,24 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>New York Rangers</t>
+          <t>Winnipeg Jets</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>89.1225</v>
+        <v>88.723</v>
       </c>
       <c r="F25" t="n">
-        <v>13.40335251852586</v>
+        <v>13.01841076713629</v>
       </c>
       <c r="G25" t="n">
         <v>67</v>
@@ -2383,45 +2383,45 @@
         <v>89</v>
       </c>
       <c r="I25" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J25" t="n">
-        <v>0.3395</v>
+        <v>0.3758</v>
       </c>
       <c r="K25" t="n">
-        <v>0.0522</v>
+        <v>0.0346</v>
       </c>
       <c r="L25" t="n">
-        <v>0.0233</v>
+        <v>0.0236</v>
       </c>
       <c r="M25" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0108</v>
       </c>
       <c r="N25" t="n">
-        <v>7.823147646950697</v>
+        <v>8.140000216729245</v>
       </c>
       <c r="O25" t="n">
-        <v>8.699999999999999</v>
+        <v>-0.8</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>+11011</t>
+          <t>+9159</t>
         </is>
       </c>
       <c r="Q25" t="n">
-        <v>-4.799844584438726</v>
+        <v>-2.74817447802685</v>
       </c>
       <c r="R25" t="n">
-        <v>-1.908540197038762</v>
+        <v>-0.03608817469521482</v>
       </c>
       <c r="S25" t="n">
-        <v>0.4458023315861614</v>
+        <v>-2.183910751078082</v>
       </c>
       <c r="T25" t="n">
-        <v>-0.1363557253125856</v>
+        <v>1.080791714011119</v>
       </c>
       <c r="U25" t="n">
-        <v>0.8318037149568038</v>
+        <v>0.09443943429775073</v>
       </c>
     </row>
     <row r="26">
@@ -2444,13 +2444,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>87.82940000000001</v>
+        <v>88.6086</v>
       </c>
       <c r="F26" t="n">
-        <v>13.27973383668051</v>
+        <v>13.22873032345119</v>
       </c>
       <c r="G26" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H26" t="n">
         <v>88</v>
@@ -2459,16 +2459,16 @@
         <v>110</v>
       </c>
       <c r="J26" t="n">
-        <v>0.3901</v>
+        <v>0.4084</v>
       </c>
       <c r="K26" t="n">
-        <v>0.0617</v>
+        <v>0.0684</v>
       </c>
       <c r="L26" t="n">
-        <v>0.024</v>
+        <v>0.0252</v>
       </c>
       <c r="M26" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0092</v>
       </c>
       <c r="N26" t="n">
         <v>6.925373482467831</v>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>+12558</t>
+          <t>+10770</t>
         </is>
       </c>
       <c r="Q26" t="n">
@@ -2517,31 +2517,31 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>86.32299999999999</v>
+        <v>86.8292</v>
       </c>
       <c r="F27" t="n">
-        <v>13.2306982483017</v>
+        <v>13.18876118906435</v>
       </c>
       <c r="G27" t="n">
         <v>65</v>
       </c>
       <c r="H27" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I27" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J27" t="n">
-        <v>0.2575</v>
+        <v>0.2694</v>
       </c>
       <c r="K27" t="n">
-        <v>0.027</v>
+        <v>0.0292</v>
       </c>
       <c r="L27" t="n">
-        <v>0.0152</v>
+        <v>0.0159</v>
       </c>
       <c r="M27" t="n">
-        <v>0.0051</v>
+        <v>0.0054</v>
       </c>
       <c r="N27" t="n">
         <v>7.181298352106282</v>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>+19508</t>
+          <t>+18419</t>
         </is>
       </c>
       <c r="Q27" t="n">
@@ -2590,13 +2590,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>86.06999999999999</v>
+        <v>85.6073</v>
       </c>
       <c r="F28" t="n">
-        <v>13.05300494498525</v>
+        <v>13.035132457241</v>
       </c>
       <c r="G28" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H28" t="n">
         <v>86</v>
@@ -2605,16 +2605,16 @@
         <v>107</v>
       </c>
       <c r="J28" t="n">
-        <v>0.3378</v>
+        <v>0.3232</v>
       </c>
       <c r="K28" t="n">
-        <v>0.047</v>
+        <v>0.0435</v>
       </c>
       <c r="L28" t="n">
-        <v>0.0179</v>
+        <v>0.0188</v>
       </c>
       <c r="M28" t="n">
-        <v>0.0066</v>
+        <v>0.0077</v>
       </c>
       <c r="N28" t="n">
         <v>7.118157267955309</v>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>+15052</t>
+          <t>+12887</t>
         </is>
       </c>
       <c r="Q28" t="n">
@@ -2663,13 +2663,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>84.5046</v>
+        <v>84.2174</v>
       </c>
       <c r="F29" t="n">
-        <v>13.2016441090009</v>
+        <v>13.15804129211732</v>
       </c>
       <c r="G29" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H29" t="n">
         <v>84</v>
@@ -2678,16 +2678,16 @@
         <v>106</v>
       </c>
       <c r="J29" t="n">
-        <v>0.2955</v>
+        <v>0.2855</v>
       </c>
       <c r="K29" t="n">
-        <v>0.0382</v>
+        <v>0.0359</v>
       </c>
       <c r="L29" t="n">
-        <v>0.0138</v>
+        <v>0.0129</v>
       </c>
       <c r="M29" t="n">
-        <v>0.0053</v>
+        <v>0.0041</v>
       </c>
       <c r="N29" t="n">
         <v>5.794809968760188</v>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>+18768</t>
+          <t>+24290</t>
         </is>
       </c>
       <c r="Q29" t="n">
@@ -2736,10 +2736,10 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>83.2178</v>
+        <v>83.2413</v>
       </c>
       <c r="F30" t="n">
-        <v>13.17292358406345</v>
+        <v>13.1236998388315</v>
       </c>
       <c r="G30" t="n">
         <v>62</v>
@@ -2751,16 +2751,16 @@
         <v>105</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1958</v>
+        <v>0.1942</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0185</v>
+        <v>0.0197</v>
       </c>
       <c r="L30" t="n">
-        <v>0.0094</v>
+        <v>0.0101</v>
       </c>
       <c r="M30" t="n">
-        <v>0.0037</v>
+        <v>0.0039</v>
       </c>
       <c r="N30" t="n">
         <v>5.904979974439156</v>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>+26927</t>
+          <t>+25541</t>
         </is>
       </c>
       <c r="Q30" t="n">
@@ -2795,71 +2795,71 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chicago Blackhawks</t>
+          <t>Calgary Flames</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>80.64570000000001</v>
+        <v>81.1888</v>
       </c>
       <c r="F31" t="n">
-        <v>13.13801477595551</v>
+        <v>12.92486207918586</v>
       </c>
       <c r="G31" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H31" t="n">
         <v>81</v>
       </c>
       <c r="I31" t="n">
-        <v>102.0499999999993</v>
+        <v>103</v>
       </c>
       <c r="J31" t="n">
-        <v>0.1786</v>
+        <v>0.2039</v>
       </c>
       <c r="K31" t="n">
-        <v>0.0095</v>
+        <v>0.0221</v>
       </c>
       <c r="L31" t="n">
-        <v>0.0053</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="M31" t="n">
-        <v>0.0024</v>
+        <v>0.0031</v>
       </c>
       <c r="N31" t="n">
-        <v>6.748602304917045</v>
+        <v>4.091492155309823</v>
       </c>
       <c r="O31" t="n">
-        <v>11.4</v>
+        <v>-0.6</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>+41567</t>
+          <t>+32158</t>
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>-14.08048256211883</v>
+        <v>-7.566996579698094</v>
       </c>
       <c r="R31" t="n">
-        <v>-0.4221108765379712</v>
+        <v>-0.1681206183302957</v>
       </c>
       <c r="S31" t="n">
-        <v>2.496371645999701</v>
+        <v>0.4355320155673481</v>
       </c>
       <c r="T31" t="n">
-        <v>-0.8766338907976194</v>
+        <v>-0.9345974485237442</v>
       </c>
       <c r="U31" t="n">
-        <v>-1.025233403433248</v>
+        <v>-3.769962061404637</v>
       </c>
     </row>
     <row r="32">
@@ -2868,71 +2868,71 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Calgary Flames</t>
+          <t>Chicago Blackhawks</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>80.34690000000001</v>
+        <v>81.0604</v>
       </c>
       <c r="F32" t="n">
-        <v>12.98744885544414</v>
+        <v>13.08781421506635</v>
       </c>
       <c r="G32" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H32" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I32" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J32" t="n">
-        <v>0.1905</v>
+        <v>0.1828</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0212</v>
+        <v>0.0106</v>
       </c>
       <c r="L32" t="n">
-        <v>0.0086</v>
+        <v>0.0065</v>
       </c>
       <c r="M32" t="n">
-        <v>0.003</v>
+        <v>0.0026</v>
       </c>
       <c r="N32" t="n">
-        <v>4.091492155309823</v>
+        <v>6.748602304917045</v>
       </c>
       <c r="O32" t="n">
-        <v>-0.6</v>
+        <v>11.4</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>+33233</t>
+          <t>+38362</t>
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>-7.566996579698094</v>
+        <v>-14.08048256211883</v>
       </c>
       <c r="R32" t="n">
-        <v>-0.1681206183302957</v>
+        <v>-0.4221108765379712</v>
       </c>
       <c r="S32" t="n">
-        <v>0.4355320155673481</v>
+        <v>2.496371645999701</v>
       </c>
       <c r="T32" t="n">
-        <v>-0.9345974485237442</v>
+        <v>-0.8766338907976194</v>
       </c>
       <c r="U32" t="n">
-        <v>-3.769962061404637</v>
+        <v>-1.025233403433248</v>
       </c>
     </row>
     <row r="33">
@@ -2955,31 +2955,31 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>78.35809999999999</v>
+        <v>78.5949</v>
       </c>
       <c r="F33" t="n">
-        <v>12.89331951666505</v>
+        <v>12.86193363859775</v>
       </c>
       <c r="G33" t="n">
         <v>57</v>
       </c>
       <c r="H33" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I33" t="n">
         <v>99</v>
       </c>
       <c r="J33" t="n">
-        <v>0.1563</v>
+        <v>0.1592</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0136</v>
+        <v>0.0128</v>
       </c>
       <c r="L33" t="n">
-        <v>0.0054</v>
+        <v>0.0049</v>
       </c>
       <c r="M33" t="n">
-        <v>0.0018</v>
+        <v>0.0015</v>
       </c>
       <c r="N33" t="n">
         <v>5.049701439462</v>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>+55456</t>
+          <t>+66567</t>
         </is>
       </c>
       <c r="Q33" t="n">

</xml_diff>